<commit_message>
Corregge la cancellazione dei dati con la sincronizzazione attiva
Cancellare in locale non bastava: al primo allineamento l'archivio condiviso
rimandava indietro tutto, e i dati sembravano non sparire mai.

- 'Cancella i dati' ora distingue fra solo su questo dispositivo (che spegne
  anche la sincronizzazione, altrimenti il problema si ripresenta) e su tutti i
  dispositivi, che svuota anche l'archivio condiviso
- la cancellazione globale trasforma i record in lapidi con data recente, cosi
  vincono sulle copie degli altri dispositivi e li svuotano a loro volta
- opzione per conservare nome negozio, fornitore e aliquota predefinita
- le lapidi piu vecchie di 90 giorni vengono scartate al caricamento
- esempio-prodotti.xlsx: 32 articoli, tre aliquote (22/10/4), margini coerenti

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/esempio-prodotti.xlsx
+++ b/esempio-prodotti.xlsx
@@ -433,15 +433,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -592,7 +592,7 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>22</v>
@@ -630,27 +630,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Candela cera di soia lavanda</t>
+          <t>Ciondolo vetro di Murano</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CAN-10</t>
+          <t>CIO-06</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>9.9</v>
+        <v>27</v>
       </c>
       <c r="D7" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Casa</t>
+          <t>Bigiotteria</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>24</v>
+        <v>66</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>22</v>
@@ -659,27 +659,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Candela cera di soia agrumi</t>
+          <t>Fermacapelli legno</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAN-11</t>
+          <t>FER-07</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>9.9</v>
+        <v>7.5</v>
       </c>
       <c r="D8" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Casa</t>
+          <t>Bigiotteria</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>22</v>
@@ -688,19 +688,19 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Diffusore vimini 100 ml</t>
+          <t>Candela soia lavanda</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>DIF-12</t>
+          <t>CAN-10</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>17.5</v>
+        <v>9.9</v>
       </c>
       <c r="D9" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -708,7 +708,7 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="G9" s="3" t="n">
         <v>22</v>
@@ -717,19 +717,19 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Tazza ceramica smaltata</t>
+          <t>Candela soia agrumi</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>TAZ-13</t>
+          <t>CAN-11</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>12</v>
+        <v>9.9</v>
       </c>
       <c r="D10" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="G10" s="3" t="n">
         <v>22</v>
@@ -746,27 +746,27 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ciotola gres media</t>
+          <t>Candela soia legno di cedro</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CIO-14</t>
+          <t>CAN-12</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="D11" t="n">
         <v>15</v>
       </c>
-      <c r="D11" t="n">
-        <v>8</v>
-      </c>
       <c r="E11" t="inlineStr">
         <is>
           <t>Casa</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="G11" s="3" t="n">
         <v>22</v>
@@ -775,19 +775,19 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Vassoio legno ulivo</t>
+          <t>Diffusore vimini 100 ml</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>VAS-15</t>
+          <t>DIF-13</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>28</v>
+        <v>17.5</v>
       </c>
       <c r="D12" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -795,7 +795,7 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>68</v>
+        <v>42</v>
       </c>
       <c r="G12" s="3" t="n">
         <v>22</v>
@@ -804,27 +804,27 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Sciarpa lana merino</t>
+          <t>Tazza ceramica smaltata</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SCI-20</t>
+          <t>TAZ-14</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="D13" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Tessuti</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>85</v>
+        <v>29</v>
       </c>
       <c r="G13" s="3" t="n">
         <v>22</v>
@@ -833,27 +833,27 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sciarpa cotone leggera</t>
+          <t>Ciotola gres media</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>SCI-21</t>
+          <t>CIT-15</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="D14" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Tessuti</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="G14" s="3" t="n">
         <v>22</v>
@@ -862,27 +862,27 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Borsa tela stampata</t>
+          <t>Vassoio legno ulivo</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>BOR-22</t>
+          <t>VAS-16</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>19.5</v>
+        <v>28</v>
       </c>
       <c r="D15" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Tessuti</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="G15" s="3" t="n">
         <v>22</v>
@@ -891,27 +891,27 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Pochette lino ricamata</t>
+          <t>Portacandele ferro battuto</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>POC-23</t>
+          <t>POR-17</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Tessuti</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="G16" s="3" t="n">
         <v>22</v>
@@ -920,27 +920,27 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Grembiule cucina</t>
+          <t>Set 2 tovagliette lino</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>GRE-24</t>
+          <t>TOV-18</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D17" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Tessuti</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="G17" s="3" t="n">
         <v>22</v>
@@ -949,27 +949,27 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Quaderno rilegato a mano</t>
+          <t>Sciarpa lana merino</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>QUA-30</t>
+          <t>SCI-20</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>8.5</v>
+        <v>35</v>
       </c>
       <c r="D18" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Cartoleria</t>
+          <t>Tessuti</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>21</v>
+        <v>85</v>
       </c>
       <c r="G18" s="3" t="n">
         <v>22</v>
@@ -978,27 +978,27 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Set 5 cartoline illustrate</t>
+          <t>Sciarpa cotone leggera</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CAR-31</t>
+          <t>SCI-21</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="D19" t="n">
         <v>6</v>
       </c>
-      <c r="D19" t="n">
-        <v>20</v>
-      </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Cartoleria</t>
+          <t>Tessuti</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>15</v>
+        <v>54</v>
       </c>
       <c r="G19" s="3" t="n">
         <v>22</v>
@@ -1007,27 +1007,27 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Segnalibro ottone</t>
+          <t>Borsa tela stampata</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>SEG-32</t>
+          <t>BOR-22</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>5.5</v>
+        <v>19.5</v>
       </c>
       <c r="D20" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Cartoleria</t>
+          <t>Tessuti</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>14</v>
+        <v>48</v>
       </c>
       <c r="G20" s="3" t="n">
         <v>22</v>
@@ -1036,30 +1036,378 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>Pochette lino ricamata</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>POC-23</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="D21" t="n">
+        <v>8</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Tessuti</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Grembiule cucina</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>GRE-24</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="D22" t="n">
+        <v>5</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Tessuti</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Cappello lana cotta</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>CAP-25</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="D23" t="n">
+        <v>4</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Tessuti</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Quaderno rilegato a mano</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>QUA-30</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D24" t="n">
+        <v>15</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Cartoleria</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Set 5 cartoline illustrate</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>CAR-31</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D25" t="n">
+        <v>20</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Cartoleria</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="G25" s="3" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Segnalibro ottone</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>SEG-32</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="D26" t="n">
+        <v>18</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Cartoleria</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="G26" s="3" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Calendario da tavolo</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>CAL-33</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="D27" t="n">
+        <v>10</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Cartoleria</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>Guida illustrata della citta</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>GUI-33</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="n">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>GUI-34</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="D21" t="n">
+      <c r="D28" t="n">
+        <v>12</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Cartoleria</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="G28" s="3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Ricettario tradizioni locali</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>RIC-35</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D29" t="n">
+        <v>8</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Cartoleria</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="G29" s="3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Confettura albicocche 220 g</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>CNF-40</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="D30" t="n">
+        <v>24</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Gastronomia</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="G30" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Cartoleria</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="n">
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Miele di acacia 250 g</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>MIE-41</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="D31" t="n">
+        <v>24</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Gastronomia</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="G31" s="3" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Biscotti di mais 200 g</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>BIS-42</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="D32" t="n">
+        <v>30</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Gastronomia</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="G32" s="3" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Tisana erbe di montagna</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>TIS-43</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="D33" t="n">
         <v>18</v>
       </c>
-      <c r="G21" s="3" t="n">
-        <v>4</v>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Gastronomia</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="G33" s="3" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>